<commit_message>
Add checkout field validation tests
</commit_message>
<xml_diff>
--- a/src/test/java/test-cases-scenarios/Checkout-Test-cases.xlsx
+++ b/src/test/java/test-cases-scenarios/Checkout-Test-cases.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18420" windowHeight="6720"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -321,12 +322,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -341,11 +348,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -626,7 +634,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -637,7 +645,7 @@
     <col min="6" max="6" width="107.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -660,7 +668,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -679,8 +687,9 @@
       <c r="G2" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -699,8 +708,9 @@
       <c r="G3" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -719,8 +729,9 @@
       <c r="G4" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -739,8 +750,9 @@
       <c r="G5" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -759,8 +771,9 @@
       <c r="G6" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -779,8 +792,9 @@
       <c r="G7" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -799,8 +813,9 @@
       <c r="G8" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -819,8 +834,9 @@
       <c r="G9" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -839,8 +855,9 @@
       <c r="G10" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>35</v>
       </c>
@@ -860,7 +877,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -880,7 +897,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>40</v>
       </c>
@@ -900,7 +917,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -920,7 +937,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -940,7 +957,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>49</v>
       </c>

</xml_diff>

<commit_message>
Update checkout test scenarios
</commit_message>
<xml_diff>
--- a/src/test/java/test-cases-scenarios/Checkout-Test-cases.xlsx
+++ b/src/test/java/test-cases-scenarios/Checkout-Test-cases.xlsx
@@ -4,13 +4,12 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18420" windowHeight="6720"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="108">
   <si>
     <t xml:space="preserve">TC ID </t>
   </si>
@@ -70,15 +69,9 @@
     <t>CHK-003</t>
   </si>
   <si>
-    <t>Shipping Address zorunlu alanlarının boş bırakılması</t>
-  </si>
-  <si>
     <t>Shipping Address formu açık</t>
   </si>
   <si>
-    <t>Zorunlu alanların her biri için kendi validation mesajı görüntülenir</t>
-  </si>
-  <si>
     <t>CHK-004</t>
   </si>
   <si>
@@ -145,30 +138,15 @@
     <t>CHK-012</t>
   </si>
   <si>
-    <t>Address 1 minimum karakter sınırının doğrulanması</t>
-  </si>
-  <si>
     <t>Address 1 validation mesajı görüntülenir</t>
   </si>
   <si>
     <t>CHK-013</t>
   </si>
   <si>
-    <t>City minimum karakter sınırının doğrulanması</t>
-  </si>
-  <si>
-    <t>City validation mesajı görüntülenir</t>
-  </si>
-  <si>
     <t>CHK-014</t>
   </si>
   <si>
-    <t>Post Code karakter sınırının doğrulanması</t>
-  </si>
-  <si>
-    <t>Post Code validation mesajı görüntülenir</t>
-  </si>
-  <si>
     <t>CHK-015</t>
   </si>
   <si>
@@ -190,9 +168,6 @@
     <t>1. Shipping Method bölümündeki Choose butonuna tıkla</t>
   </si>
   <si>
-    <t>CHK-017</t>
-  </si>
-  <si>
     <t>Shipping Address tamamlandıktan sonra Shipping Method seçimi</t>
   </si>
   <si>
@@ -203,9 +178,6 @@
   </si>
   <si>
     <t>Kullanılabilir Shipping Method seçenekleri görüntülenir</t>
-  </si>
-  <si>
-    <t>CHK-018</t>
   </si>
   <si>
     <t>Shipping Method seçilmeden checkout akışına devam edilmesi</t>
@@ -231,10 +203,6 @@
   <si>
     <t>1. Basket sayfasına git
 2. Checkout butonuna tıkla</t>
-  </si>
-  <si>
-    <t>1. Tüm alanları boş bırak
-2. Continue'a tıkla</t>
   </si>
   <si>
     <t>1. First Name'i boş bırak
@@ -265,23 +233,6 @@
     <t>1. Region/State alanında seçim yapma
 2. Diğer zorunlu alanları geçerli doldur
 3. Continue'a tıkla</t>
-  </si>
-  <si>
-    <t>1. First Name'e 32 karakterden fazla değer gir
-2. Continue'a tıkla</t>
-  </si>
-  <si>
-    <t>1. Address 1'e 3 karakterden kısa değer gir
-2. Diğer alanları geçerli doldur
-3. Continue'a tıkla</t>
-  </si>
-  <si>
-    <t>1. City alanına 2 karakterden kısa değer gir
-2. Continue'a tıkla</t>
-  </si>
-  <si>
-    <t>1. Post Code'a 2 karakterden kısa veya 10 karakterden uzun değer gir
-2. Continue'a tıkla</t>
   </si>
   <si>
     <t>1. First Name gir
@@ -308,13 +259,200 @@
   <si>
     <t>Negative</t>
   </si>
+  <si>
+    <t>Boundry</t>
+  </si>
+  <si>
+    <t>1. First Name'e 32 karakterden fazla değer gir:33
+2. Continue'a tıkla</t>
+  </si>
+  <si>
+    <t>First Name validation mesajı görüntülenmez</t>
+  </si>
+  <si>
+    <t>Address 129 maksimum  karakter sınırının doğrulanması</t>
+  </si>
+  <si>
+    <t>1. Address 1 e 129 karakter gir.
+2. Diğer alanları geçerli doldur
+3. Continue'a tıkla</t>
+  </si>
+  <si>
+    <t>Negative Boundry</t>
+  </si>
+  <si>
+    <t>Geçerli Shipping Address bilgileri ile adresin başarıyla kaydedilmesi</t>
+  </si>
+  <si>
+    <t>Kullanıcı giriş yapmış olmalı ve sepette ürün bulunmalı. Checkout sayfasında yeni adres seçilmeli.</t>
+  </si>
+  <si>
+    <t>1. Checkout sayfasına git.
+2. New Address seçeneğini seç.
+3. First Name alanına geçerli değer gir.
+4. Last Name alanına geçerli değer gir.
+5. Address 1 alanına geçerli değer gir.
+6. City alanına geçerli değer gir.
+7. Post Code alanına geçerli değer gir.
+8. Country seç.
+9. Region/State seç.
+10. Continue butonuna tıkla.</t>
+  </si>
+  <si>
+    <t>First Name: A
+Last Name: Test
+Address 1: Test Address
+City: Istanbul
+Post Code: 34000
+Country: United Kingdom
+Region: Bristol</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> "Success: You have changed shipping address!" alert mesajı görüntülenir. </t>
+  </si>
+  <si>
+    <t>Deneme1@gmail.com Deneme1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yeni kayıtşı data oluşturmak zorunlu </t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test1</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test2</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test3</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test4</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test5</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test6</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test7</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test8</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test9</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test10</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test11</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test12</t>
+  </si>
+  <si>
+    <t>Test1@gmail.com Test13</t>
+  </si>
+  <si>
+    <t>Kayıtlı adres bulunmayan kullanıcı için Shipping Method seçimi</t>
+  </si>
+  <si>
+    <t>Kayıtlı adres bulunan kullanıcı için New Address ile Shipping Method seçimi</t>
+  </si>
+  <si>
+    <t>Kayıtlı adres bulunan kullanıcı için mevcut adresi kullanarak Shipping Method seçimi</t>
+  </si>
+  <si>
+    <t>Kullanıcı giriş yapmış, sepette ürün var, kayıtlı shipping address yok</t>
+  </si>
+  <si>
+    <t>Kullanıcı giriş yapmış, kayıtlı shipping address mevcut, sepette ürün var</t>
+  </si>
+  <si>
+    <t>1. Checkout'a git
+2. Shipping Address bilgilerini doldur
+3. Shipping Address → Continue
+4. Shipping Method → Choose
+5. Flat Shipping Rate seçili gelir
+6. Continue'a bas</t>
+  </si>
+  <si>
+    <t>1. Checkout'a git
+2. New Address seç
+3. Shipping Address bilgilerini doldur
+4. Continue
+5. Shipping Method → Choose
+6. Flat Shipping Rate seçili gelir
+1. Checkout'a git
+2. New Address seç
+3. Shipping Address bilgilerini doldur
+4. Continue
+5. Shipping Method → Choose
+6. Flat Shipping Rate seçili gelir
+7. Continue</t>
+  </si>
+  <si>
+    <t>1. Checkout'a git
+2. Kayıtlı adresi seç
+3. Shipping Address → Continue
+4. Shipping Method → Choose
+5. Flat Shipping Rate seçili gelir
+6. Continue</t>
+  </si>
+  <si>
+    <t>Shipping Method başarıyla kaydedilir ve Checkout sayfasındaki Shipping Method alanında Flat Shipping Rate - $8.00 görüntülenir</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Shipping Method başarıyla kaydedilir ve Checkout sayfasındaki Shipping Method alanında </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Flat Shipping Rate - $8.00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> görüntülenir</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -345,17 +483,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Köprü" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -634,15 +775,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="64.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="80.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="107.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="107.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -679,15 +821,18 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="G2" t="s">
-        <v>84</v>
-      </c>
-      <c r="H2" s="2"/>
+        <v>70</v>
+      </c>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -702,343 +847,416 @@
       <c r="D3" t="s">
         <v>13</v>
       </c>
+      <c r="E3" t="s">
+        <v>84</v>
+      </c>
       <c r="F3" t="s">
         <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>84</v>
-      </c>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>15</v>
       </c>
       <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>70</v>
+        <v>61</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>85</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="G4" t="s">
-        <v>85</v>
-      </c>
-      <c r="H4" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
         <v>71</v>
       </c>
-      <c r="F5" t="s">
-        <v>65</v>
-      </c>
-      <c r="G5" t="s">
-        <v>85</v>
-      </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>72</v>
+        <v>63</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="F6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>85</v>
-      </c>
-      <c r="H6" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>73</v>
+        <v>64</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G7" t="s">
-        <v>85</v>
-      </c>
-      <c r="H7" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="H7" s="3"/>
     </row>
     <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>74</v>
+        <v>65</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>89</v>
       </c>
       <c r="F8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>85</v>
-      </c>
-      <c r="H8" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="H8" s="3"/>
     </row>
     <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>75</v>
+        <v>66</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="F9" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="G9" t="s">
-        <v>85</v>
-      </c>
-      <c r="H9" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="H9" s="3"/>
     </row>
     <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
         <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F10" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" t="s">
+        <v>72</v>
+      </c>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F11" t="s">
+        <v>35</v>
+      </c>
+      <c r="G11" t="s">
+        <v>72</v>
+      </c>
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F10" t="s">
-        <v>66</v>
-      </c>
-      <c r="G10" t="s">
-        <v>85</v>
-      </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F11" t="s">
-        <v>37</v>
-      </c>
-      <c r="G11" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="E12" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" t="s">
+        <v>77</v>
+      </c>
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>38</v>
       </c>
-      <c r="B12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F12" t="s">
-        <v>37</v>
-      </c>
-      <c r="G12" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F13" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>40</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14" t="s">
+        <v>58</v>
+      </c>
+      <c r="G14" t="s">
+        <v>71</v>
+      </c>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>41</v>
       </c>
-      <c r="C13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="1" t="s">
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" t="s">
+        <v>70</v>
+      </c>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F16" t="s">
+        <v>59</v>
+      </c>
+      <c r="G16" t="s">
+        <v>71</v>
+      </c>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" spans="1:8" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" t="s">
         <v>78</v>
       </c>
-      <c r="F13" t="s">
-        <v>42</v>
-      </c>
-      <c r="G13" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>43</v>
-      </c>
-      <c r="B14" t="s">
-        <v>44</v>
-      </c>
-      <c r="C14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="1" t="s">
+      <c r="C17" t="s">
         <v>79</v>
       </c>
-      <c r="F14" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>46</v>
-      </c>
-      <c r="B15" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="1" t="s">
+      <c r="D17" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F15" t="s">
-        <v>48</v>
-      </c>
-      <c r="G15" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F16" t="s">
-        <v>51</v>
-      </c>
-      <c r="G16" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>52</v>
-      </c>
-      <c r="B17" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" t="s">
-        <v>54</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F17" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="G17" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>56</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="H17" s="3"/>
+    </row>
+    <row r="18" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>57</v>
+        <v>98</v>
       </c>
       <c r="C18" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
       <c r="F18" t="s">
-        <v>60</v>
+        <v>107</v>
       </c>
       <c r="G18" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>61</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="H18" s="3"/>
+    </row>
+    <row r="19" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
-        <v>62</v>
+        <v>99</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>102</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="F19" t="s">
-        <v>68</v>
+        <v>107</v>
       </c>
       <c r="G19" t="s">
-        <v>85</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="H19" s="3"/>
+    </row>
+    <row r="20" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" t="s">
+        <v>102</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F20" t="s">
+        <v>106</v>
+      </c>
+      <c r="G20" t="s">
+        <v>70</v>
+      </c>
+      <c r="H20" s="3"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1"/>
+    <hyperlink ref="E4" r:id="rId2"/>
+    <hyperlink ref="E5:E11" r:id="rId3" display="Test1@gmail.com Test1"/>
+    <hyperlink ref="E12" r:id="rId4" display="Test1@gmail.com Test1"/>
+    <hyperlink ref="E13:E16" r:id="rId5" display="Test1@gmail.com Test1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>